<commit_message>
Fixing logic errors in bom and KEV loading
</commit_message>
<xml_diff>
--- a/examples/template.xlsx
+++ b/examples/template.xlsx
@@ -122,7 +122,7 @@
     <t xml:space="preserve">Residual Risk Scoring Details</t>
   </si>
   <si>
-    <t xml:space="preserve">Safety Heatmap</t>
+    <t xml:space="preserve">Cyber to Safety Heat-Map</t>
   </si>
   <si>
     <t xml:space="preserve">Column Name</t>
@@ -140,13 +140,13 @@
     <t xml:space="preserve">Negligible</t>
   </si>
   <si>
-    <t xml:space="preserve">Minor</t>
+    <t xml:space="preserve">Minor / Marginal</t>
   </si>
   <si>
     <t xml:space="preserve">Serious</t>
   </si>
   <si>
-    <t xml:space="preserve">Critical/Catastrophic</t>
+    <t xml:space="preserve">Critical / Catastrophic</t>
   </si>
   <si>
     <t xml:space="preserve">Attack Vector (AV)</t>
@@ -158,19 +158,19 @@
     <t xml:space="preserve">Critical</t>
   </si>
   <si>
+    <t xml:space="preserve">Uncontrolled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack Complexity (AC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low (0.77), High (0.44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
     <t xml:space="preserve">Controlled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncontrolled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attack Complexity (AC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low (0.77), High (0.44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
   </si>
   <si>
     <t xml:space="preserve">Privileges Required (PR)</t>
@@ -260,42 +260,12 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF729FCF"/>
-        <bgColor rgb="FF969696"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE0C2CD"/>
-        <bgColor rgb="FFFFCCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF5CE"/>
-        <bgColor rgb="FFE8F2A1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F2A1"/>
-        <bgColor rgb="FFFFF5CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFA6A6"/>
-        <bgColor rgb="FFE0C2CD"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -305,8 +275,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDEDCE6"/>
+        <bgColor rgb="FFFFD7D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF5CE"/>
+        <bgColor rgb="FFF6F9D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F9D4"/>
+        <bgColor rgb="FFFFF5CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD7D7"/>
+        <bgColor rgb="FFFFCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFDBB6"/>
-        <bgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFFFD7D7"/>
       </patternFill>
     </fill>
   </fills>
@@ -351,7 +345,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -420,40 +414,36 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -469,7 +459,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF729FCF"/>
+          <fgColor rgb="FFB4C7DC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -484,7 +474,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE0C2CD"/>
+          <fgColor rgb="FFDEDCE6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -508,7 +498,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE8F2A1"/>
+          <fgColor rgb="FFF6F9D4"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -516,7 +506,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFA6A6"/>
+          <fgColor rgb="FFFFD7D7"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -551,7 +541,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFF5CE"/>
       <rgbColor rgb="FFCC0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -566,14 +556,14 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFB4C7DC"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF729FCF"/>
+      <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF5CE"/>
+      <rgbColor rgb="FFF6F9D4"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFE0C2CD"/>
+      <rgbColor rgb="FFDEDCE6"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -585,9 +575,9 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFE8F2A1"/>
+      <rgbColor rgb="FFFFD7D7"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFFA6A6"/>
+      <rgbColor rgb="FFFFCCCC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFDBB6"/>
       <rgbColor rgb="FF3366FF"/>
@@ -1052,17 +1042,17 @@
       <c r="F4" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="25" t="s">
-        <v>45</v>
+      <c r="H4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1070,29 +1060,29 @@
         <v>18</v>
       </c>
       <c r="B5" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>46</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>47</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F5" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="J5" s="13" t="s">
         <v>44</v>
-      </c>
-      <c r="I5" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1112,17 +1102,17 @@
       <c r="F6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="13" t="s">
         <v>44</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" s="25" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1142,16 +1132,16 @@
       <c r="F7" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" s="25" t="s">
+      <c r="G7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="13" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1208,6 +1198,16 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="E2:J2"/>
   </mergeCells>
+  <conditionalFormatting sqref="G4:J7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"Controlled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:J7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>"Uncontrolled"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add certificate flag and correct minor errors
</commit_message>
<xml_diff>
--- a/examples/template.xlsx
+++ b/examples/template.xlsx
@@ -1042,16 +1042,16 @@
       <c r="F4" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1072,16 +1072,16 @@
       <c r="F5" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="J5" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1102,16 +1102,16 @@
       <c r="F6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="J6" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1132,16 +1132,16 @@
       <c r="F7" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1202,8 +1202,6 @@
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Controlled"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:J7">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Uncontrolled"</formula>
     </cfRule>

</xml_diff>